<commit_message>
updated portals, state, and cleanup logic
</commit_message>
<xml_diff>
--- a/Users.xlsx
+++ b/Users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\PR\Imperial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C75BBFC8-06E1-4F08-8122-9A637404DDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C5D826-FE90-41F3-80BF-ED16F282051C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Directors" sheetId="1" r:id="rId1"/>
@@ -30,14 +30,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="92">
   <si>
     <t xml:space="preserve">Sr </t>
   </si>
   <si>
-    <t xml:space="preserve">Name </t>
-  </si>
-  <si>
     <t xml:space="preserve">Email </t>
   </si>
   <si>
@@ -53,9 +50,6 @@
     <t xml:space="preserve">Ishwari Deshmukh </t>
   </si>
   <si>
-    <t xml:space="preserve">ishwari.deshmukh@gmail.com </t>
-  </si>
-  <si>
     <t>Shrikrishna Deshmukh</t>
   </si>
   <si>
@@ -264,13 +258,61 @@
   </si>
   <si>
     <t>Per subject 10,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee details per subject </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Students name </t>
+  </si>
+  <si>
+    <t>99217 98749</t>
+  </si>
+  <si>
+    <t>788 766 3080</t>
+  </si>
+  <si>
+    <t>90211 30871</t>
+  </si>
+  <si>
+    <t>87998 69325</t>
+  </si>
+  <si>
+    <t>724 922 7159</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 94222 93946</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 98234 55980</t>
+  </si>
+  <si>
+    <t>87673 89453</t>
+  </si>
+  <si>
+    <t>724 922 7158</t>
+  </si>
+  <si>
+    <t>724 922 7157</t>
+  </si>
+  <si>
+    <t>Name of Teacher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of Admin </t>
+  </si>
+  <si>
+    <t>Name of Directors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ishwari1.deshmukh@gmail.com </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -285,12 +327,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color rgb="FF334155"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -314,10 +350,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -614,19 +649,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -634,10 +669,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>9850311082</v>
@@ -648,10 +683,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D4">
         <v>9823979878</v>
@@ -684,19 +719,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -704,10 +739,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>9850311082</v>
@@ -745,28 +780,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -774,110 +809,110 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>9823283377</v>
       </c>
       <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
         <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C3" s="1"/>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
         <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="I5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
         <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
         <v>17</v>
-      </c>
-      <c r="H7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" t="s">
         <v>17</v>
-      </c>
-      <c r="H8" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s">
         <v>17</v>
-      </c>
-      <c r="H9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I9" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -885,66 +920,66 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2">
+        <v>9</v>
+      </c>
+      <c r="D12">
         <v>9370728283</v>
       </c>
       <c r="G12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I13" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -952,77 +987,77 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="G17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
         <v>31</v>
-      </c>
-      <c r="D17" t="s">
-        <v>32</v>
-      </c>
-      <c r="G17" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" t="s">
-        <v>18</v>
-      </c>
-      <c r="I17" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H20" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G22" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -1030,44 +1065,44 @@
         <v>4</v>
       </c>
       <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G23" t="s">
+        <v>26</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="s">
         <v>35</v>
-      </c>
-      <c r="C23" t="s">
-        <v>38</v>
-      </c>
-      <c r="D23" t="s">
-        <v>36</v>
-      </c>
-      <c r="G23" t="s">
-        <v>28</v>
-      </c>
-      <c r="H23" t="s">
-        <v>18</v>
-      </c>
-      <c r="I23" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G24" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H24" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G25" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H25" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1088,7 +1123,8 @@
   <cols>
     <col min="1" max="1" width="2.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.26953125" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.36328125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1098,28 +1134,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1127,19 +1163,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2" t="s">
-        <v>41</v>
-      </c>
       <c r="I2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -1147,30 +1186,33 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" t="s">
-        <v>43</v>
-      </c>
-      <c r="I3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -1178,74 +1220,77 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
+      </c>
+      <c r="D5" t="s">
+        <v>80</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -1253,19 +1298,22 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>81</v>
       </c>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -1273,30 +1321,33 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" t="s">
+        <v>49</v>
+      </c>
+      <c r="I12" t="s">
         <v>50</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G12" t="s">
-        <v>40</v>
-      </c>
-      <c r="H12" t="s">
-        <v>51</v>
-      </c>
-      <c r="I12" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H13" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13" t="s">
         <v>51</v>
-      </c>
-      <c r="I13" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1319,6 +1370,8 @@
     <col min="1" max="1" width="3.08984375" customWidth="1"/>
     <col min="2" max="2" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.08984375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -1329,31 +1382,31 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
       <c r="H1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -1361,22 +1414,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="H2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I2" t="s">
-        <v>41</v>
-      </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -1384,33 +1440,36 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" t="s">
         <v>42</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" t="s">
-        <v>40</v>
-      </c>
-      <c r="I3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -1418,77 +1477,80 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
+      </c>
+      <c r="E5" t="s">
+        <v>85</v>
       </c>
       <c r="H5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -1496,22 +1558,25 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>87</v>
       </c>
       <c r="H11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="J11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1519,33 +1584,36 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
+        <v>86</v>
+      </c>
+      <c r="H12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" t="s">
         <v>50</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I12" t="s">
-        <v>51</v>
-      </c>
-      <c r="J12" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I13" t="s">
+        <v>49</v>
+      </c>
+      <c r="J13" t="s">
         <v>51</v>
-      </c>
-      <c r="J13" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1562,132 +1630,137 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECCE93A3-D131-49A5-AA8E-E9200EB09E87}">
-  <dimension ref="A2:B18"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>76</v>
+      </c>
+    </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>